<commit_message>
feat: Izinkan penentuan Nomor Ujian manual dari file Excel saat import siswa
</commit_message>
<xml_diff>
--- a/file_testing/template_data_siswa_ekonomika.xlsx
+++ b/file_testing/template_data_siswa_ekonomika.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G15"/>
+  <dimension ref="A1:H6"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -416,337 +416,148 @@
         <v>Tanggal Lahir</v>
       </c>
       <c r="F1" t="str">
+        <v>Nomor Ujian</v>
+      </c>
+      <c r="G1" t="str">
         <v>Ruang Ujian</v>
       </c>
-      <c r="G1" t="str">
+      <c r="H1" t="str">
         <v>Password Ujian</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>101000001</v>
+        <v>0011223301</v>
       </c>
       <c r="B2" t="str">
-        <v>AHMAD SANTOSO</v>
+        <v>AHMAD SUBARJO</v>
       </c>
       <c r="C2" t="str">
-        <v xml:space="preserve">X AKL </v>
+        <v>X AKL</v>
       </c>
       <c r="D2" t="str">
-        <v>Jakarta</v>
+        <v>DEPOK</v>
       </c>
       <c r="E2" t="str">
-        <v>2010-01-15</v>
+        <v>2008-01-15</v>
       </c>
       <c r="F2" t="str">
-        <v>001</v>
+        <v>U-X-AKL-001</v>
       </c>
       <c r="G2" t="str">
-        <v>xakl123</v>
+        <v>R-01</v>
+      </c>
+      <c r="H2" t="str">
+        <v>pass01</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>101000002</v>
+        <v>0011223302</v>
       </c>
       <c r="B3" t="str">
-        <v>BUDI SETIAWAN</v>
+        <v>BUDI SANTOSO</v>
       </c>
       <c r="C3" t="str">
         <v>X DKV</v>
       </c>
       <c r="D3" t="str">
-        <v>Bogor</v>
+        <v>JAKARTA</v>
       </c>
       <c r="E3" t="str">
-        <v>2010-02-20</v>
+        <v>2008-02-20</v>
       </c>
       <c r="F3" t="str">
-        <v>001</v>
+        <v>U-X-DKV-001</v>
       </c>
       <c r="G3" t="str">
-        <v>xdkv123</v>
+        <v>R-02</v>
+      </c>
+      <c r="H3" t="str">
+        <v>pass02</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>101000003</v>
+        <v>0011223303</v>
       </c>
       <c r="B4" t="str">
-        <v>CHIKA AMALIA</v>
+        <v>CITRA LESTARI</v>
       </c>
       <c r="C4" t="str">
         <v>X PH 1</v>
       </c>
       <c r="D4" t="str">
-        <v>Depok</v>
+        <v>BOGOR</v>
       </c>
       <c r="E4" t="str">
-        <v>2010-03-25</v>
+        <v>2008-03-25</v>
       </c>
       <c r="F4" t="str">
-        <v>002</v>
+        <v>U-X-PH1-001</v>
       </c>
       <c r="G4" t="str">
-        <v>xph123</v>
+        <v>R-03</v>
+      </c>
+      <c r="H4" t="str">
+        <v>pass03</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>101000004</v>
+        <v>0011223304</v>
       </c>
       <c r="B5" t="str">
-        <v>DEWI LESTARI</v>
+        <v>DINA MARIANA</v>
       </c>
       <c r="C5" t="str">
-        <v>X PH 2</v>
+        <v>XI MPLB</v>
       </c>
       <c r="D5" t="str">
-        <v>Tangerang</v>
+        <v>TANGERANG</v>
       </c>
       <c r="E5" t="str">
-        <v>2010-04-10</v>
+        <v>2007-04-10</v>
       </c>
       <c r="F5" t="str">
-        <v>002</v>
+        <v>U-XI-MPLB-001</v>
       </c>
       <c r="G5" t="str">
-        <v>xph456</v>
+        <v>R-04</v>
+      </c>
+      <c r="H5" t="str">
+        <v>pass04</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>101000005</v>
+        <v>0011223305</v>
       </c>
       <c r="B6" t="str">
         <v>EKO PRASETYO</v>
       </c>
       <c r="C6" t="str">
-        <v>X MPLB</v>
+        <v>XII AKL</v>
       </c>
       <c r="D6" t="str">
-        <v>Bekasi</v>
+        <v>BEKASI</v>
       </c>
       <c r="E6" t="str">
-        <v>2010-05-05</v>
+        <v>2006-05-05</v>
       </c>
       <c r="F6" t="str">
-        <v>003</v>
+        <v>U-XII-AKL-001</v>
       </c>
       <c r="G6" t="str">
-        <v>xmplb123</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v>111000001</v>
-      </c>
-      <c r="B7" t="str">
-        <v>FAHRI ZAINUDIN</v>
-      </c>
-      <c r="C7" t="str">
-        <v>XI DEKUNTAN</v>
-      </c>
-      <c r="D7" t="str">
-        <v>Jakarta</v>
-      </c>
-      <c r="E7" t="str">
-        <v>2009-06-12</v>
-      </c>
-      <c r="F7" t="str">
-        <v>004</v>
-      </c>
-      <c r="G7" t="str">
-        <v>xidek123</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="str">
-        <v>111000002</v>
-      </c>
-      <c r="B8" t="str">
-        <v>GITA WIRJAWAN</v>
-      </c>
-      <c r="C8" t="str">
-        <v xml:space="preserve">XI MPLB </v>
-      </c>
-      <c r="D8" t="str">
-        <v>Bandung</v>
-      </c>
-      <c r="E8" t="str">
-        <v>2009-07-18</v>
-      </c>
-      <c r="F8" t="str">
-        <v>004</v>
-      </c>
-      <c r="G8" t="str">
-        <v>ximplb123</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="str">
-        <v>111000003</v>
-      </c>
-      <c r="B9" t="str">
-        <v>HARI DARMAWAN</v>
-      </c>
-      <c r="C9" t="str">
-        <v>XI PH</v>
-      </c>
-      <c r="D9" t="str">
-        <v>Surabaya</v>
-      </c>
-      <c r="E9" t="str">
-        <v>2009-08-22</v>
-      </c>
-      <c r="F9" t="str">
-        <v>005</v>
-      </c>
-      <c r="G9" t="str">
-        <v>xiph123</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="str">
-        <v>121000001</v>
-      </c>
-      <c r="B10" t="str">
-        <v>INTAN PERMATA</v>
-      </c>
-      <c r="C10" t="str">
-        <v>XII MPLB 1</v>
-      </c>
-      <c r="D10" t="str">
-        <v>Semarang</v>
-      </c>
-      <c r="E10" t="str">
-        <v>2008-09-30</v>
-      </c>
-      <c r="F10" t="str">
-        <v>006</v>
-      </c>
-      <c r="G10" t="str">
-        <v>xiimplb123</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="str">
-        <v>121000002</v>
-      </c>
-      <c r="B11" t="str">
-        <v>JOKO SUSILO</v>
-      </c>
-      <c r="C11" t="str">
-        <v>XII MPLB 2</v>
-      </c>
-      <c r="D11" t="str">
-        <v>Yogyakarta</v>
-      </c>
-      <c r="E11" t="str">
-        <v>2008-10-14</v>
-      </c>
-      <c r="F11" t="str">
-        <v>006</v>
-      </c>
-      <c r="G11" t="str">
-        <v>xiimplb456</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="str">
-        <v>121000003</v>
-      </c>
-      <c r="B12" t="str">
-        <v>KARTIKA SARI</v>
-      </c>
-      <c r="C12" t="str">
-        <v>XII PH 1</v>
-      </c>
-      <c r="D12" t="str">
-        <v>Malang</v>
-      </c>
-      <c r="E12" t="str">
-        <v>2008-11-09</v>
-      </c>
-      <c r="F12" t="str">
-        <v>007</v>
-      </c>
-      <c r="G12" t="str">
-        <v>xiiph123</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="str">
-        <v>121000004</v>
-      </c>
-      <c r="B13" t="str">
-        <v>LUKMAN HAKIM</v>
-      </c>
-      <c r="C13" t="str">
-        <v>XII PH 2</v>
-      </c>
-      <c r="D13" t="str">
-        <v>Surakarta</v>
-      </c>
-      <c r="E13" t="str">
-        <v>2008-12-01</v>
-      </c>
-      <c r="F13" t="str">
-        <v>007</v>
-      </c>
-      <c r="G13" t="str">
-        <v>xiiph456</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="str">
-        <v>121000005</v>
-      </c>
-      <c r="B14" t="str">
-        <v>MIA KHALIDA</v>
-      </c>
-      <c r="C14" t="str">
-        <v>XII AKL</v>
-      </c>
-      <c r="D14" t="str">
-        <v>Cirebon</v>
-      </c>
-      <c r="E14" t="str">
-        <v>2008-01-20</v>
-      </c>
-      <c r="F14" t="str">
-        <v>008</v>
-      </c>
-      <c r="G14" t="str">
-        <v>xiiakl123</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="str">
-        <v>121000006</v>
-      </c>
-      <c r="B15" t="str">
-        <v>NANDA SAPUTRA</v>
-      </c>
-      <c r="C15" t="str">
-        <v>XII DKV</v>
-      </c>
-      <c r="D15" t="str">
-        <v>Tasikmalaya</v>
-      </c>
-      <c r="E15" t="str">
-        <v>2008-02-28</v>
-      </c>
-      <c r="F15" t="str">
-        <v>008</v>
-      </c>
-      <c r="G15" t="str">
-        <v>xiidkv123</v>
+        <v>R-05</v>
+      </c>
+      <c r="H6" t="str">
+        <v>pass05</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G15"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H6"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>